<commit_message>
Fix: ajustes api send, faq, lancamentos e modelo importacao
</commit_message>
<xml_diff>
--- a/public/modelo_importacao_cartao-credito.xlsx
+++ b/public/modelo_importacao_cartao-credito.xlsx
@@ -19,6 +19,7 @@
     <definedName name="Administrativo">Informações!$J$92:$J$95</definedName>
     <definedName name="Alimentação">Informações!$J$2:$J$6</definedName>
     <definedName name="Assinaturas_e_Serviços">Informações!$J$7:$J$11</definedName>
+    <definedName name="Bem_estar">Informações!$J$12:$J$16</definedName>
     <definedName name="Compras">Informações!$J$12:$J$17</definedName>
     <definedName name="Condomínio_Despesa">Informações!$G$19:$G$22</definedName>
     <definedName name="Condomínio_Receita">Informações!$G$29:$G$30</definedName>
@@ -56,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="166">
   <si>
     <t>banco</t>
   </si>
@@ -538,7 +539,22 @@
     <t>Março/2026</t>
   </si>
   <si>
-    <t>Veículo Aplicativo</t>
+    <t>Bem estar</t>
+  </si>
+  <si>
+    <t>Salão de beleza</t>
+  </si>
+  <si>
+    <t>Estética</t>
+  </si>
+  <si>
+    <t>Spa/Massagem</t>
+  </si>
+  <si>
+    <t>Barbearia</t>
+  </si>
+  <si>
+    <t>Salão de Beleza</t>
   </si>
 </sst>
 </file>
@@ -1214,16 +1230,16 @@
         <v>46082</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="G4" s="21" t="s">
         <v>159</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>29</v>
+        <v>160</v>
       </c>
       <c r="I4" s="19" t="s">
-        <v>79</v>
+        <v>161</v>
       </c>
       <c r="J4" s="19">
         <v>125</v>
@@ -6019,7 +6035,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A1:AA113"/>
+  <dimension ref="A1:AA118"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.5703125" style="2" customWidth="1"/>
@@ -6222,7 +6238,7 @@
         <v>149</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>23</v>
+        <v>160</v>
       </c>
       <c r="I4" s="9" t="s">
         <v>15</v>
@@ -6231,7 +6247,7 @@
         <v>47</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>23</v>
+        <v>160</v>
       </c>
       <c r="N4" s="15" t="s">
         <v>15</v>
@@ -6269,7 +6285,7 @@
         <v>149</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I5" s="9" t="s">
         <v>15</v>
@@ -6278,7 +6294,7 @@
         <v>48</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="N5" s="15" t="s">
         <v>15</v>
@@ -6316,7 +6332,7 @@
         <v>149</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I6" s="9" t="s">
         <v>15</v>
@@ -6325,7 +6341,7 @@
         <v>30</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="N6" s="15" t="s">
         <v>15</v>
@@ -6361,7 +6377,7 @@
         <v>149</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I7" s="9" t="s">
         <v>84</v>
@@ -6370,7 +6386,7 @@
         <v>50</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N7" s="15" t="s">
         <v>84</v>
@@ -6400,7 +6416,7 @@
         <v>149</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I8" s="9" t="s">
         <v>84</v>
@@ -6409,7 +6425,7 @@
         <v>51</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N8" s="15" t="s">
         <v>84</v>
@@ -6437,7 +6453,7 @@
         <v>149</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I9" s="9" t="s">
         <v>84</v>
@@ -6446,7 +6462,7 @@
         <v>52</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N9" s="15" t="s">
         <v>84</v>
@@ -6474,7 +6490,7 @@
         <v>149</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I10" s="9" t="s">
         <v>84</v>
@@ -6483,7 +6499,7 @@
         <v>53</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N10" s="15" t="s">
         <v>84</v>
@@ -6511,7 +6527,7 @@
         <v>149</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I11" s="9" t="s">
         <v>84</v>
@@ -6520,7 +6536,7 @@
         <v>30</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N11" s="15" t="s">
         <v>84</v>
@@ -6548,22 +6564,22 @@
         <v>149</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>23</v>
+        <v>160</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>54</v>
+        <v>161</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="N12" s="15" t="s">
-        <v>23</v>
+        <v>160</v>
       </c>
       <c r="O12" s="15" t="s">
-        <v>54</v>
+        <v>161</v>
       </c>
       <c r="Q12"/>
       <c r="S12" s="4" t="s">
@@ -6582,22 +6598,25 @@
     </row>
     <row r="13" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F13" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>33</v>
+        <v>83</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>23</v>
+        <v>160</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>55</v>
+        <v>164</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>83</v>
       </c>
       <c r="N13" s="15" t="s">
-        <v>23</v>
+        <v>160</v>
       </c>
       <c r="O13" s="15" t="s">
-        <v>55</v>
+        <v>164</v>
       </c>
       <c r="Q13"/>
       <c r="S13" s="4" t="s">
@@ -6619,19 +6638,19 @@
         <v>150</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>23</v>
+        <v>160</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>56</v>
+        <v>162</v>
       </c>
       <c r="N14" s="15" t="s">
-        <v>23</v>
+        <v>160</v>
       </c>
       <c r="O14" s="15" t="s">
-        <v>56</v>
+        <v>162</v>
       </c>
       <c r="Q14"/>
       <c r="S14" s="4" t="s">
@@ -6653,19 +6672,19 @@
         <v>150</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>23</v>
+        <v>160</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>57</v>
+        <v>163</v>
       </c>
       <c r="N15" s="15" t="s">
-        <v>23</v>
+        <v>160</v>
       </c>
       <c r="O15" s="15" t="s">
-        <v>57</v>
+        <v>163</v>
       </c>
       <c r="Q15"/>
       <c r="S15" s="4" t="s">
@@ -6687,19 +6706,19 @@
         <v>150</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>23</v>
+        <v>160</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="N16" s="15" t="s">
-        <v>23</v>
+        <v>160</v>
       </c>
       <c r="O16" s="15" t="s">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="Q16"/>
       <c r="S16" s="4" t="s">
@@ -6721,19 +6740,19 @@
         <v>150</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I17" s="9" t="s">
         <v>23</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="N17" s="15" t="s">
         <v>23</v>
       </c>
       <c r="O17" s="15" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="Q17"/>
       <c r="S17" s="4" t="s">
@@ -6755,19 +6774,19 @@
         <v>150</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="N18" s="15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O18" s="15" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="Q18"/>
       <c r="S18" s="4" t="s">
@@ -6786,22 +6805,22 @@
     </row>
     <row r="19" spans="6:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F19" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="N19" s="15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O19" s="15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="Q19"/>
       <c r="S19" s="4" t="s">
@@ -6816,19 +6835,19 @@
         <v>151</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="N20" s="15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O20" s="15" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="Q20"/>
       <c r="S20" s="4" t="s">
@@ -6852,19 +6871,19 @@
         <v>151</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>44</v>
+        <v>120</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="N21" s="15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O21" s="15" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="Q21"/>
       <c r="S21" s="4" t="s">
@@ -6888,19 +6907,19 @@
         <v>151</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="N22" s="15" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O22" s="15" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="Q22"/>
       <c r="S22" s="4" t="s">
@@ -6918,22 +6937,22 @@
     </row>
     <row r="23" spans="6:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F23" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="G23" s="15" t="s">
-        <v>142</v>
+        <v>151</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>45</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="N23" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O23" s="15" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="Q23"/>
       <c r="S23" s="4" t="s">
@@ -6954,19 +6973,19 @@
         <v>146</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J24" s="9" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N24" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O24" s="15" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="Q24"/>
       <c r="S24" s="4" t="s">
@@ -6987,19 +7006,19 @@
         <v>146</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="N25" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O25" s="15" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="Q25"/>
       <c r="S25" s="4" t="s">
@@ -7020,19 +7039,19 @@
         <v>146</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="N26" s="15" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="O26" s="15" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="Q26"/>
       <c r="S26" s="4" t="s">
@@ -7053,19 +7072,19 @@
         <v>146</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="N27" s="15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O27" s="15" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="Q27"/>
       <c r="S27" s="4" t="s">
@@ -7083,22 +7102,22 @@
     </row>
     <row r="28" spans="6:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F28" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>137</v>
+        <v>146</v>
+      </c>
+      <c r="G28" s="15" t="s">
+        <v>140</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J28" s="9" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="N28" s="15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O28" s="15" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="Q28"/>
       <c r="S28" s="4" t="s">
@@ -7110,22 +7129,22 @@
     </row>
     <row r="29" spans="6:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F29" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J29" s="9" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="N29" s="15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O29" s="15" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="30" spans="6:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7133,16 +7152,16 @@
         <v>148</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I30" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J30" s="9" t="s">
         <v>30</v>
       </c>
       <c r="N30" s="15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O30" s="15" t="s">
         <v>30</v>
@@ -7158,17 +7177,23 @@
       </c>
     </row>
     <row r="31" spans="6:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F31" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>139</v>
+      </c>
       <c r="I31" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J31" s="9" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="N31" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O31" s="15" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="S31" s="4" t="s">
         <v>137</v>
@@ -7178,17 +7203,23 @@
       </c>
     </row>
     <row r="32" spans="6:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F32" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>139</v>
+      </c>
       <c r="I32" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J32" s="9" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="N32" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O32" s="15" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="S32" s="4" t="s">
         <v>137</v>
@@ -7199,16 +7230,16 @@
     </row>
     <row r="33" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I33" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J33" s="9" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="N33" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O33" s="15" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="S33" s="4" t="s">
         <v>137</v>
@@ -7219,30 +7250,30 @@
     </row>
     <row r="34" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I34" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J34" s="9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="N34" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O34" s="15" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="35" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I35" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J35" s="9" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="N35" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O35" s="15" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7250,13 +7281,13 @@
         <v>27</v>
       </c>
       <c r="J36" s="9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N36" s="15" t="s">
         <v>27</v>
       </c>
       <c r="O36" s="15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="37" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7264,13 +7295,13 @@
         <v>27</v>
       </c>
       <c r="J37" s="9" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="N37" s="15" t="s">
         <v>27</v>
       </c>
       <c r="O37" s="15" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7278,616 +7309,646 @@
         <v>27</v>
       </c>
       <c r="J38" s="9" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="N38" s="15" t="s">
         <v>27</v>
       </c>
       <c r="O38" s="15" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I39" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J39" s="9" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="N39" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O39" s="15" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="40" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I40" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J40" s="9" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="N40" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O40" s="15" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="41" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I41" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J41" s="9" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="N41" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O41" s="15" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="42" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I42" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J42" s="9" t="s">
-        <v>30</v>
+        <v>74</v>
       </c>
       <c r="N42" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O42" s="15" t="s">
-        <v>30</v>
+        <v>74</v>
       </c>
     </row>
     <row r="43" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I43" s="9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J43" s="9" t="s">
-        <v>78</v>
+        <v>30</v>
       </c>
       <c r="N43" s="15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="O43" s="15" t="s">
-        <v>78</v>
+        <v>30</v>
       </c>
     </row>
     <row r="44" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I44" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J44" s="9" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="N44" s="15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O44" s="15" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="45" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I45" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J45" s="9" t="s">
-        <v>43</v>
+        <v>76</v>
       </c>
       <c r="N45" s="15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O45" s="15" t="s">
-        <v>43</v>
+        <v>76</v>
       </c>
     </row>
     <row r="46" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I46" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J46" s="9" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="N46" s="15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O46" s="15" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
     </row>
     <row r="47" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I47" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="J47" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="J47" s="9" t="s">
-        <v>80</v>
-      </c>
       <c r="N47" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="O47" s="15" t="s">
         <v>30</v>
-      </c>
-      <c r="O47" s="15" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="48" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I48" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J48" s="9" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="N48" s="15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O48" s="15" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="49" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I49" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J49" s="9" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="N49" s="15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O49" s="15" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="50" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I50" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J50" s="9" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="N50" s="15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O50" s="15" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
     </row>
     <row r="51" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I51" s="9" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="J51" s="9" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="N51" s="15" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="O51" s="15" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
     </row>
     <row r="52" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I52" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="J52" s="14" t="s">
-        <v>86</v>
+      <c r="I52" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="J52" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="N52" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="O52" s="15" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="53" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I53" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="J53" s="14" t="s">
-        <v>87</v>
+      <c r="I53" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="J53" s="9" t="s">
+        <v>81</v>
       </c>
       <c r="L53" s="15" t="s">
         <v>142</v>
       </c>
       <c r="N53" s="15" t="s">
-        <v>142</v>
+        <v>30</v>
       </c>
       <c r="O53" s="15" t="s">
-        <v>107</v>
+        <v>81</v>
       </c>
     </row>
     <row r="54" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I54" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="J54" s="14" t="s">
-        <v>88</v>
+      <c r="I54" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="J54" s="9" t="s">
+        <v>82</v>
       </c>
       <c r="L54" s="15" t="s">
         <v>143</v>
       </c>
       <c r="N54" s="15" t="s">
-        <v>142</v>
+        <v>30</v>
       </c>
       <c r="O54" s="15" t="s">
-        <v>108</v>
+        <v>82</v>
       </c>
     </row>
     <row r="55" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I55" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="J55" s="14" t="s">
-        <v>89</v>
+      <c r="I55" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="J55" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="L55" s="15" t="s">
         <v>144</v>
       </c>
       <c r="N55" s="15" t="s">
-        <v>142</v>
+        <v>30</v>
       </c>
       <c r="O55" s="15" t="s">
-        <v>109</v>
+        <v>30</v>
       </c>
     </row>
     <row r="56" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I56" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="J56" s="14" t="s">
-        <v>30</v>
+      <c r="I56" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="J56" s="9" t="s">
+        <v>83</v>
       </c>
       <c r="L56" s="15" t="s">
         <v>145</v>
       </c>
       <c r="N56" s="15" t="s">
-        <v>142</v>
+        <v>83</v>
       </c>
       <c r="O56" s="15" t="s">
-        <v>110</v>
+        <v>83</v>
       </c>
     </row>
     <row r="57" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I57" s="8" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="J57" s="14" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="L57" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="N57" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="O57" s="15" t="s">
-        <v>30</v>
-      </c>
     </row>
     <row r="58" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I58" s="8" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="J58" s="14" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="L58"/>
       <c r="N58" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O58" s="15" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="59" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I59" s="8" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="J59" s="14" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="L59"/>
       <c r="N59" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O59" s="15" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="60" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I60" s="8" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="J60" s="14" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="L60"/>
       <c r="N60" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O60" s="15" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="61" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I61" s="8" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="J61" s="14" t="s">
         <v>30</v>
       </c>
       <c r="L61"/>
       <c r="N61" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O61" s="15" t="s">
-        <v>30</v>
+        <v>110</v>
       </c>
     </row>
     <row r="62" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I62" s="8" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="J62" s="14" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="L62"/>
       <c r="N62" s="15" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O62" s="15" t="s">
-        <v>114</v>
+        <v>30</v>
       </c>
     </row>
     <row r="63" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I63" s="8" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="J63" s="14" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="L63"/>
       <c r="N63" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O63" s="15" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="64" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I64" s="8" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="J64" s="14" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="L64"/>
       <c r="N64" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O64" s="15" t="s">
-        <v>30</v>
+        <v>112</v>
       </c>
     </row>
     <row r="65" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I65" s="8" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="J65" s="14" t="s">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="L65"/>
       <c r="N65" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="O65" s="15" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="66" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I66" s="8" t="s">
-        <v>35</v>
+        <v>85</v>
       </c>
       <c r="J66" s="14" t="s">
-        <v>97</v>
+        <v>30</v>
       </c>
       <c r="L66"/>
       <c r="N66" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="O66" s="15" t="s">
-        <v>117</v>
+        <v>30</v>
       </c>
     </row>
     <row r="67" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I67" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J67" s="14" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="L67"/>
       <c r="N67" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O67" s="15" t="s">
-        <v>30</v>
+        <v>114</v>
       </c>
     </row>
     <row r="68" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I68" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J68" s="14" t="s">
-        <v>52</v>
+        <v>95</v>
       </c>
       <c r="L68"/>
       <c r="N68" s="15" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="O68" s="15" t="s">
-        <v>141</v>
+        <v>115</v>
       </c>
     </row>
     <row r="69" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I69" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J69" s="14" t="s">
-        <v>43</v>
+        <v>96</v>
       </c>
       <c r="L69"/>
       <c r="N69" s="15" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="O69" s="15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="70" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I70" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J70" s="14" t="s">
         <v>30</v>
       </c>
       <c r="L70"/>
       <c r="N70" s="15" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="O70" s="15" t="s">
-        <v>30</v>
+        <v>116</v>
       </c>
     </row>
     <row r="71" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I71" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J71" s="14" t="s">
-        <v>98</v>
+        <v>97</v>
+      </c>
+      <c r="N71" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="O71" s="15" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="72" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I72" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J72" s="14" t="s">
-        <v>99</v>
+        <v>72</v>
+      </c>
+      <c r="N72" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="O72" s="15" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="73" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I73" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J73" s="14" t="s">
-        <v>100</v>
+        <v>52</v>
+      </c>
+      <c r="N73" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="O73" s="15" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="74" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I74" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J74" s="14" t="s">
-        <v>30</v>
+        <v>43</v>
+      </c>
+      <c r="N74" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="O74" s="15" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="75" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I75" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="J75" s="14" t="s">
-        <v>101</v>
+        <v>30</v>
+      </c>
+      <c r="N75" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="O75" s="15" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="76" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I76" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J76" s="14" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="77" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I77" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J77" s="14" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="78" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I78" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="J78" s="14" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="79" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I79" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="J79" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="80" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I80" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="J78" s="14" t="s">
+      <c r="J80" s="14" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="81" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I81" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J81" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="82" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I82" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J82" s="14" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="83" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I83" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J83" s="14" t="s">
         <v>30</v>
-      </c>
-    </row>
-    <row r="79" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I79" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="J79" s="13" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="80" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I80" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="J80" s="13" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="81" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I81" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="J81" s="13" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="82" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I82" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="J82" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="83" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I83" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="J83" s="13" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="84" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I84" s="12" t="s">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="J84" s="13" t="s">
-        <v>122</v>
+        <v>90</v>
       </c>
     </row>
     <row r="85" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I85" s="12" t="s">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="J85" s="13" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="86" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I86" s="12" t="s">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="J86" s="13" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="87" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I87" s="12" t="s">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="J87" s="13" t="s">
         <v>30</v>
@@ -7895,209 +7956,249 @@
     </row>
     <row r="88" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I88" s="12" t="s">
-        <v>44</v>
+        <v>120</v>
       </c>
       <c r="J88" s="13" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="89" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I89" s="12" t="s">
-        <v>44</v>
+        <v>120</v>
       </c>
       <c r="J89" s="13" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="90" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I90" s="12" t="s">
-        <v>44</v>
+        <v>120</v>
       </c>
       <c r="J90" s="13" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="91" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I91" s="12" t="s">
-        <v>44</v>
+        <v>120</v>
       </c>
       <c r="J91" s="13" t="s">
-        <v>30</v>
+        <v>124</v>
       </c>
     </row>
     <row r="92" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I92" s="12" t="s">
-        <v>45</v>
+        <v>120</v>
       </c>
       <c r="J92" s="13" t="s">
-        <v>128</v>
+        <v>30</v>
       </c>
     </row>
     <row r="93" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I93" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J93" s="13" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="94" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I94" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J94" s="13" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="95" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I95" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="J95" s="13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="96" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I96" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="J96" s="13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="97" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I97" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="J95" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="96" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I96" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="J96" s="15" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="97" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I97" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="J97" s="15" t="s">
-        <v>108</v>
+      <c r="J97" s="13" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="98" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I98" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="J98" s="15" t="s">
-        <v>109</v>
+      <c r="I98" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="J98" s="13" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="99" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I99" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="J99" s="15" t="s">
-        <v>110</v>
+      <c r="I99" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="J99" s="13" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="100" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I100" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="J100" s="15" t="s">
+      <c r="I100" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="J100" s="13" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="101" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I101" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J101" s="15" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="102" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I102" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J102" s="15" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="103" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I103" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J103" s="15" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="104" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I104" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J104" s="15" t="s">
-        <v>30</v>
+        <v>110</v>
       </c>
     </row>
     <row r="105" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I105" s="15" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J105" s="15" t="s">
-        <v>114</v>
+        <v>30</v>
       </c>
     </row>
     <row r="106" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I106" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J106" s="15" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="107" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I107" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J107" s="15" t="s">
-        <v>30</v>
+        <v>112</v>
       </c>
     </row>
     <row r="108" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I108" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J108" s="15" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="109" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I109" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J109" s="15" t="s">
-        <v>117</v>
+        <v>30</v>
       </c>
     </row>
     <row r="110" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I110" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J110" s="15" t="s">
-        <v>30</v>
+        <v>114</v>
       </c>
     </row>
     <row r="111" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I111" s="15" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="J111" s="15" t="s">
-        <v>141</v>
+        <v>115</v>
       </c>
     </row>
     <row r="112" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I112" s="15" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="J112" s="15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="113" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I113" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="J113" s="15" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="114" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I114" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="J114" s="15" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="115" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I115" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="J115" s="15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="116" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I116" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="J113" s="15" t="s">
+      <c r="J116" s="15" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="117" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I117" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="J117" s="15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="118" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I118" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="J118" s="15" t="s">
         <v>30</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: ajustes modelo importacao debito e credito
</commit_message>
<xml_diff>
--- a/public/modelo_importacao_cartao-credito.xlsx
+++ b/public/modelo_importacao_cartao-credito.xlsx
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="166">
   <si>
     <t>banco</t>
   </si>
@@ -7203,12 +7203,6 @@
       </c>
     </row>
     <row r="32" spans="6:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F32" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="G32" s="4" t="s">
-        <v>139</v>
-      </c>
       <c r="I32" s="9" t="s">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
Fix: ajustes lancamentos e modelo importacao
</commit_message>
<xml_diff>
--- a/public/modelo_importacao_cartao-credito.xlsx
+++ b/public/modelo_importacao_cartao-credito.xlsx
@@ -20,44 +20,45 @@
     <definedName name="Alimentação">Informações!$J$2:$J$6</definedName>
     <definedName name="Assinaturas_e_Serviços">Informações!$J$7:$J$11</definedName>
     <definedName name="Bem_estar">Informações!$J$12:$J$16</definedName>
-    <definedName name="Compras">Informações!$J$12:$J$17</definedName>
-    <definedName name="Condomínio_Despesa">Informações!$G$19:$G$22</definedName>
-    <definedName name="Condomínio_Receita">Informações!$G$29:$G$30</definedName>
+    <definedName name="Compras">Informações!$J$17:$J$22</definedName>
+    <definedName name="Condomínio_Despesa">Informações!$G$21:$G$24</definedName>
+    <definedName name="Condomínio_Receita">Informações!$G$31:$G$32</definedName>
     <definedName name="Despesa">Informações!$D$5:$D$7</definedName>
-    <definedName name="Educação">Informações!$J$18:$J$21</definedName>
-    <definedName name="Empresarial_Despesa">Informações!$G$13:$G$18</definedName>
-    <definedName name="Empresarial_Receita">Informações!$G$28</definedName>
-    <definedName name="Financeiro">Informações!$J$75:$J$78</definedName>
-    <definedName name="Folha_de_Pagamento">Informações!$J$79:$J$82</definedName>
-    <definedName name="Freelance">Informações!$J$105:$J$107</definedName>
-    <definedName name="Impostos">Informações!$J$71:$J$74</definedName>
-    <definedName name="Indefinido">Informações!$J$51</definedName>
-    <definedName name="Infraestrutura">Informações!$J$66:$J$70</definedName>
-    <definedName name="Investimentos">Informações!$J$22:$J$25</definedName>
-    <definedName name="Lazer">Informações!$J$26:$J$30</definedName>
-    <definedName name="Manutenção_Condomínio">Informações!$J$83:$J$87</definedName>
-    <definedName name="Marketing">Informações!$J$62:$J$65</definedName>
-    <definedName name="Moradia">Informações!$J$31:$J$38</definedName>
-    <definedName name="Operacional">Informações!$J$52:$J$56</definedName>
-    <definedName name="Outros">Informações!$J$47:$J$50</definedName>
-    <definedName name="Pessoal_Despesa">Informações!$G$2:$G$12</definedName>
-    <definedName name="Pessoal_Empresarial">Informações!$J$57:$J$61</definedName>
-    <definedName name="Pessoal_Receita">Informações!$G$23:$G$27</definedName>
-    <definedName name="Proventos">Informações!$J$101:$J$104</definedName>
+    <definedName name="Doações">Informações!$J$23:$J$27</definedName>
+    <definedName name="Educação">Informações!$J$28:$J$31</definedName>
+    <definedName name="Empresarial_Despesa">Informações!$G$15:$G$20</definedName>
+    <definedName name="Empresarial_Receita">Informações!$G$30</definedName>
+    <definedName name="Financeiro">Informações!$J$85:$J$88</definedName>
+    <definedName name="Folha_de_Pagamento">Informações!$J$89:$J$92</definedName>
+    <definedName name="Freelance">Informações!$J$115:$J$117</definedName>
+    <definedName name="Impostos">Informações!$J$81:$J$84</definedName>
+    <definedName name="Indefinido">Informações!$J$61</definedName>
+    <definedName name="Infraestrutura">Informações!$J$76:$J$80</definedName>
+    <definedName name="Investimentos">Informações!$J$32:$J$35</definedName>
+    <definedName name="Lazer">Informações!$J$36:$J$40</definedName>
+    <definedName name="Manutenção_Condomínio">Informações!$J$93:$J$97</definedName>
+    <definedName name="Marketing">Informações!$J$72:$J$75</definedName>
+    <definedName name="Moradia">Informações!$J$41:$J$48</definedName>
+    <definedName name="Operacional">Informações!$J$62:$J$66</definedName>
+    <definedName name="Outros">Informações!$J$57:$J$60</definedName>
+    <definedName name="Pessoal_Despesa">Informações!$G$2:$G$14</definedName>
+    <definedName name="Pessoal_Empresarial">Informações!$J$67:$J$71</definedName>
+    <definedName name="Pessoal_Receita">Informações!$G$25:$G$29</definedName>
+    <definedName name="Proventos">Informações!$J$111:$J$114</definedName>
     <definedName name="Receita">Informações!$D$2:$D$4</definedName>
-    <definedName name="Reembolso">Informações!$J$111:$J$113</definedName>
-    <definedName name="Salário">Informações!$J$96:$J$100</definedName>
-    <definedName name="Saúde">Informações!$J$39:$J$42</definedName>
-    <definedName name="Transporte">Informações!$J$43:$J$46</definedName>
-    <definedName name="Utilidades">Informações!$J$88:$J$91</definedName>
-    <definedName name="Vendas">Informações!$J$108:$J$110</definedName>
+    <definedName name="Reembolso">Informações!$J$121:$J$123</definedName>
+    <definedName name="Salário">Informações!$J$106:$J$110</definedName>
+    <definedName name="Saúde">Informações!$J$49:$J$52</definedName>
+    <definedName name="Transporte">Informações!$J$53:$J$56</definedName>
+    <definedName name="Utilidades">Informações!$J$98:$J$101</definedName>
+    <definedName name="Vendas">Informações!$J$118:$J$120</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="177">
   <si>
     <t>banco</t>
   </si>
@@ -555,6 +556,39 @@
   </si>
   <si>
     <t>Salão de Beleza</t>
+  </si>
+  <si>
+    <t>Bradesco</t>
+  </si>
+  <si>
+    <t>Doação</t>
+  </si>
+  <si>
+    <t>Abril/2026</t>
+  </si>
+  <si>
+    <t>Doações</t>
+  </si>
+  <si>
+    <t>Instituições de Caridade</t>
+  </si>
+  <si>
+    <t>Dízimos e Ofertas</t>
+  </si>
+  <si>
+    <t>Ajuda a Terceiros</t>
+  </si>
+  <si>
+    <t>Causas Ambientais/Animais</t>
+  </si>
+  <si>
+    <t>Itaú</t>
+  </si>
+  <si>
+    <t>Prestação Apartamento</t>
+  </si>
+  <si>
+    <t>Maio/2026</t>
   </si>
 </sst>
 </file>
@@ -1254,40 +1288,96 @@
         <v>0</v>
       </c>
       <c r="N4" s="19" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="20">
+        <v>46113</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="G5" s="21" t="s">
+        <v>168</v>
+      </c>
+      <c r="H5" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="J5" s="19">
+        <v>800</v>
+      </c>
+      <c r="K5" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="L5" s="19">
+        <v>1</v>
+      </c>
+      <c r="M5" s="19">
+        <v>3</v>
+      </c>
+      <c r="N5" s="19" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="19"/>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="21"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-    </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="19"/>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
+      <c r="A6" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="20">
+        <v>46143</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>167</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>176</v>
+      </c>
+      <c r="H6" s="19" t="s">
+        <v>169</v>
+      </c>
+      <c r="I6" s="19" t="s">
+        <v>173</v>
+      </c>
+      <c r="J6" s="19">
+        <v>50</v>
+      </c>
+      <c r="K6" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="L6" s="19">
+        <v>0</v>
+      </c>
+      <c r="M6" s="19">
+        <v>0</v>
+      </c>
+      <c r="N6" s="19" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="19"/>
@@ -1296,7 +1386,6 @@
       <c r="D7" s="19"/>
       <c r="E7" s="20"/>
       <c r="F7" s="19"/>
-      <c r="G7" s="21"/>
       <c r="H7" s="19"/>
       <c r="I7" s="19"/>
       <c r="J7" s="19"/>
@@ -6035,7 +6124,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A1:AA118"/>
+  <dimension ref="A1:AA123"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.5703125" style="2" customWidth="1"/>
@@ -6332,7 +6421,7 @@
         <v>149</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>24</v>
+        <v>169</v>
       </c>
       <c r="I6" s="9" t="s">
         <v>15</v>
@@ -6341,7 +6430,7 @@
         <v>30</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>24</v>
+        <v>169</v>
       </c>
       <c r="N6" s="15" t="s">
         <v>15</v>
@@ -6377,7 +6466,7 @@
         <v>149</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I7" s="9" t="s">
         <v>84</v>
@@ -6386,7 +6475,7 @@
         <v>50</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="N7" s="15" t="s">
         <v>84</v>
@@ -6416,7 +6505,7 @@
         <v>149</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I8" s="9" t="s">
         <v>84</v>
@@ -6425,7 +6514,7 @@
         <v>51</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N8" s="15" t="s">
         <v>84</v>
@@ -6453,7 +6542,7 @@
         <v>149</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I9" s="9" t="s">
         <v>84</v>
@@ -6462,7 +6551,7 @@
         <v>52</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N9" s="15" t="s">
         <v>84</v>
@@ -6490,7 +6579,7 @@
         <v>149</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I10" s="9" t="s">
         <v>84</v>
@@ -6499,7 +6588,7 @@
         <v>53</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N10" s="15" t="s">
         <v>84</v>
@@ -6527,7 +6616,7 @@
         <v>149</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I11" s="9" t="s">
         <v>84</v>
@@ -6536,7 +6625,7 @@
         <v>30</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N11" s="15" t="s">
         <v>84</v>
@@ -6564,7 +6653,7 @@
         <v>149</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I12" s="9" t="s">
         <v>160</v>
@@ -6573,7 +6662,7 @@
         <v>161</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N12" s="15" t="s">
         <v>160</v>
@@ -6601,7 +6690,7 @@
         <v>149</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="I13" s="9" t="s">
         <v>160</v>
@@ -6610,7 +6699,7 @@
         <v>164</v>
       </c>
       <c r="L13" s="4" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="N13" s="15" t="s">
         <v>160</v>
@@ -6635,16 +6724,19 @@
     </row>
     <row r="14" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F14" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>33</v>
+        <v>83</v>
       </c>
       <c r="I14" s="9" t="s">
         <v>160</v>
       </c>
       <c r="J14" s="9" t="s">
         <v>162</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>83</v>
       </c>
       <c r="N14" s="15" t="s">
         <v>160</v>
@@ -6672,7 +6764,7 @@
         <v>150</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="I15" s="9" t="s">
         <v>160</v>
@@ -6706,7 +6798,7 @@
         <v>150</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="I16" s="9" t="s">
         <v>160</v>
@@ -6740,7 +6832,7 @@
         <v>150</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I17" s="9" t="s">
         <v>23</v>
@@ -6774,7 +6866,7 @@
         <v>150</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I18" s="9" t="s">
         <v>23</v>
@@ -6808,7 +6900,7 @@
         <v>150</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I19" s="9" t="s">
         <v>23</v>
@@ -6832,10 +6924,10 @@
     </row>
     <row r="20" spans="6:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F20" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="I20" s="9" t="s">
         <v>23</v>
@@ -6871,7 +6963,7 @@
         <v>151</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="I21" s="9" t="s">
         <v>23</v>
@@ -6907,7 +6999,7 @@
         <v>151</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>44</v>
+        <v>120</v>
       </c>
       <c r="I22" s="9" t="s">
         <v>23</v>
@@ -6940,19 +7032,19 @@
         <v>151</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>24</v>
+        <v>169</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>59</v>
+        <v>170</v>
       </c>
       <c r="N23" s="15" t="s">
-        <v>24</v>
+        <v>169</v>
       </c>
       <c r="O23" s="15" t="s">
-        <v>59</v>
+        <v>170</v>
       </c>
       <c r="Q23"/>
       <c r="S23" s="4" t="s">
@@ -6970,22 +7062,22 @@
     </row>
     <row r="24" spans="6:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F24" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="G24" s="15" t="s">
-        <v>142</v>
+        <v>151</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>45</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>24</v>
+        <v>169</v>
       </c>
       <c r="J24" s="9" t="s">
-        <v>60</v>
+        <v>171</v>
       </c>
       <c r="N24" s="15" t="s">
-        <v>24</v>
+        <v>169</v>
       </c>
       <c r="O24" s="15" t="s">
-        <v>60</v>
+        <v>171</v>
       </c>
       <c r="Q24"/>
       <c r="S24" s="4" t="s">
@@ -7006,19 +7098,19 @@
         <v>146</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>24</v>
+        <v>169</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>61</v>
+        <v>172</v>
       </c>
       <c r="N25" s="15" t="s">
-        <v>24</v>
+        <v>169</v>
       </c>
       <c r="O25" s="15" t="s">
-        <v>61</v>
+        <v>172</v>
       </c>
       <c r="Q25"/>
       <c r="S25" s="4" t="s">
@@ -7039,19 +7131,19 @@
         <v>146</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>24</v>
+        <v>169</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>30</v>
+        <v>173</v>
       </c>
       <c r="N26" s="15" t="s">
-        <v>24</v>
+        <v>169</v>
       </c>
       <c r="O26" s="15" t="s">
-        <v>30</v>
+        <v>173</v>
       </c>
       <c r="Q26"/>
       <c r="S26" s="4" t="s">
@@ -7072,19 +7164,19 @@
         <v>146</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>25</v>
+        <v>169</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="N27" s="15" t="s">
-        <v>25</v>
+        <v>169</v>
       </c>
       <c r="O27" s="15" t="s">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="Q27"/>
       <c r="S27" s="4" t="s">
@@ -7105,19 +7197,19 @@
         <v>146</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J28" s="9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="N28" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O28" s="15" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="Q28"/>
       <c r="S28" s="4" t="s">
@@ -7129,42 +7221,42 @@
     </row>
     <row r="29" spans="6:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F29" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>137</v>
+        <v>146</v>
+      </c>
+      <c r="G29" s="15" t="s">
+        <v>140</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J29" s="9" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="N29" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O29" s="15" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="6:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F30" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I30" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J30" s="9" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="N30" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O30" s="15" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="Q30" s="4" t="s">
         <v>137</v>
@@ -7181,19 +7273,19 @@
         <v>148</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I31" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J31" s="9" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="N31" s="15" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="O31" s="15" t="s">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="S31" s="4" t="s">
         <v>137</v>
@@ -7203,17 +7295,23 @@
       </c>
     </row>
     <row r="32" spans="6:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F32" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>139</v>
+      </c>
       <c r="I32" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J32" s="9" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="N32" s="15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O32" s="15" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="S32" s="4" t="s">
         <v>137</v>
@@ -7224,16 +7322,16 @@
     </row>
     <row r="33" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I33" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J33" s="9" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="N33" s="15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O33" s="15" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="S33" s="4" t="s">
         <v>137</v>
@@ -7244,27 +7342,27 @@
     </row>
     <row r="34" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I34" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J34" s="9" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="N34" s="15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O34" s="15" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="35" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I35" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="J35" s="9" t="s">
         <v>30</v>
       </c>
       <c r="N35" s="15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O35" s="15" t="s">
         <v>30</v>
@@ -7272,72 +7370,72 @@
     </row>
     <row r="36" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I36" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J36" s="9" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="N36" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O36" s="15" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I37" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J37" s="9" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="N37" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O37" s="15" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="38" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I38" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J38" s="9" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="N38" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O38" s="15" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
     </row>
     <row r="39" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I39" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J39" s="9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="N39" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O39" s="15" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="40" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I40" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J40" s="9" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
       <c r="N40" s="15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O40" s="15" t="s">
-        <v>72</v>
+        <v>30</v>
       </c>
     </row>
     <row r="41" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7345,13 +7443,13 @@
         <v>27</v>
       </c>
       <c r="J41" s="9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="N41" s="15" t="s">
         <v>27</v>
       </c>
       <c r="O41" s="15" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="42" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7359,13 +7457,13 @@
         <v>27</v>
       </c>
       <c r="J42" s="9" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="N42" s="15" t="s">
         <v>27</v>
       </c>
       <c r="O42" s="15" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="43" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7373,616 +7471,646 @@
         <v>27</v>
       </c>
       <c r="J43" s="9" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="N43" s="15" t="s">
         <v>27</v>
       </c>
       <c r="O43" s="15" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
     </row>
     <row r="44" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I44" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J44" s="9" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="N44" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O44" s="15" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="45" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I45" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J45" s="9" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="N45" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O45" s="15" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="46" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I46" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J46" s="9" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="N46" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O46" s="15" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="47" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I47" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J47" s="9" t="s">
-        <v>30</v>
+        <v>74</v>
       </c>
       <c r="N47" s="15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O47" s="15" t="s">
-        <v>30</v>
+        <v>74</v>
       </c>
     </row>
     <row r="48" spans="9:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I48" s="9" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J48" s="9" t="s">
-        <v>78</v>
+        <v>30</v>
       </c>
       <c r="N48" s="15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="O48" s="15" t="s">
-        <v>78</v>
+        <v>30</v>
       </c>
     </row>
     <row r="49" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I49" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J49" s="9" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="N49" s="15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O49" s="15" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="50" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I50" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J50" s="9" t="s">
-        <v>43</v>
+        <v>76</v>
       </c>
       <c r="N50" s="15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O50" s="15" t="s">
-        <v>43</v>
+        <v>76</v>
       </c>
     </row>
     <row r="51" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I51" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J51" s="9" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="N51" s="15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O51" s="15" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
     </row>
     <row r="52" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I52" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="J52" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="J52" s="9" t="s">
-        <v>80</v>
-      </c>
       <c r="N52" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="O52" s="15" t="s">
         <v>30</v>
-      </c>
-      <c r="O52" s="15" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="53" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I53" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J53" s="9" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="L53" s="15" t="s">
         <v>142</v>
       </c>
       <c r="N53" s="15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O53" s="15" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="54" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I54" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J54" s="9" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="L54" s="15" t="s">
         <v>143</v>
       </c>
       <c r="N54" s="15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O54" s="15" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="55" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I55" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J55" s="9" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="L55" s="15" t="s">
         <v>144</v>
       </c>
       <c r="N55" s="15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O55" s="15" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
     </row>
     <row r="56" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I56" s="9" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="J56" s="9" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="L56" s="15" t="s">
         <v>145</v>
       </c>
       <c r="N56" s="15" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="O56" s="15" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
     </row>
     <row r="57" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I57" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="J57" s="14" t="s">
-        <v>86</v>
+      <c r="I57" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="J57" s="9" t="s">
+        <v>80</v>
       </c>
       <c r="L57" s="15" t="s">
         <v>140</v>
       </c>
+      <c r="N57" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="O57" s="15" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="58" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I58" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="J58" s="14" t="s">
-        <v>87</v>
+      <c r="I58" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="J58" s="9" t="s">
+        <v>81</v>
       </c>
       <c r="L58"/>
       <c r="N58" s="15" t="s">
-        <v>142</v>
+        <v>30</v>
       </c>
       <c r="O58" s="15" t="s">
-        <v>107</v>
+        <v>81</v>
       </c>
     </row>
     <row r="59" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I59" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="J59" s="14" t="s">
-        <v>88</v>
+      <c r="I59" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="J59" s="9" t="s">
+        <v>82</v>
       </c>
       <c r="L59"/>
       <c r="N59" s="15" t="s">
-        <v>142</v>
+        <v>30</v>
       </c>
       <c r="O59" s="15" t="s">
-        <v>108</v>
+        <v>82</v>
       </c>
     </row>
     <row r="60" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I60" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="J60" s="14" t="s">
-        <v>89</v>
+      <c r="I60" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="J60" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="L60"/>
       <c r="N60" s="15" t="s">
-        <v>142</v>
+        <v>30</v>
       </c>
       <c r="O60" s="15" t="s">
-        <v>109</v>
+        <v>30</v>
       </c>
     </row>
     <row r="61" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I61" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="J61" s="14" t="s">
-        <v>30</v>
+      <c r="I61" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="J61" s="9" t="s">
+        <v>83</v>
       </c>
       <c r="L61"/>
       <c r="N61" s="15" t="s">
-        <v>142</v>
+        <v>83</v>
       </c>
       <c r="O61" s="15" t="s">
-        <v>110</v>
+        <v>83</v>
       </c>
     </row>
     <row r="62" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I62" s="8" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="J62" s="14" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="L62"/>
-      <c r="N62" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="O62" s="15" t="s">
-        <v>30</v>
-      </c>
     </row>
     <row r="63" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I63" s="8" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="J63" s="14" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="L63"/>
       <c r="N63" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O63" s="15" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="64" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I64" s="8" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="J64" s="14" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="L64"/>
       <c r="N64" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O64" s="15" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="65" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I65" s="8" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="J65" s="14" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="L65"/>
       <c r="N65" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O65" s="15" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="66" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I66" s="8" t="s">
-        <v>85</v>
+        <v>33</v>
       </c>
       <c r="J66" s="14" t="s">
         <v>30</v>
       </c>
       <c r="L66"/>
       <c r="N66" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O66" s="15" t="s">
-        <v>30</v>
+        <v>110</v>
       </c>
     </row>
     <row r="67" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I67" s="8" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="J67" s="14" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="L67"/>
       <c r="N67" s="15" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="O67" s="15" t="s">
-        <v>114</v>
+        <v>30</v>
       </c>
     </row>
     <row r="68" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I68" s="8" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="J68" s="14" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="L68"/>
       <c r="N68" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O68" s="15" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="69" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I69" s="8" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="J69" s="14" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="L69"/>
       <c r="N69" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O69" s="15" t="s">
-        <v>30</v>
+        <v>112</v>
       </c>
     </row>
     <row r="70" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I70" s="8" t="s">
-        <v>34</v>
+        <v>85</v>
       </c>
       <c r="J70" s="14" t="s">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="L70"/>
       <c r="N70" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="O70" s="15" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="71" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I71" s="8" t="s">
-        <v>35</v>
+        <v>85</v>
       </c>
       <c r="J71" s="14" t="s">
-        <v>97</v>
+        <v>30</v>
       </c>
       <c r="N71" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="O71" s="15" t="s">
-        <v>117</v>
+        <v>30</v>
       </c>
     </row>
     <row r="72" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I72" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J72" s="14" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="N72" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="O72" s="15" t="s">
-        <v>30</v>
+        <v>114</v>
       </c>
     </row>
     <row r="73" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I73" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J73" s="14" t="s">
-        <v>52</v>
+        <v>95</v>
       </c>
       <c r="N73" s="15" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="O73" s="15" t="s">
-        <v>141</v>
+        <v>115</v>
       </c>
     </row>
     <row r="74" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I74" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J74" s="14" t="s">
-        <v>43</v>
+        <v>96</v>
       </c>
       <c r="N74" s="15" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="O74" s="15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="75" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I75" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J75" s="14" t="s">
         <v>30</v>
       </c>
       <c r="N75" s="15" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="O75" s="15" t="s">
-        <v>30</v>
+        <v>116</v>
       </c>
     </row>
     <row r="76" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I76" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J76" s="14" t="s">
-        <v>98</v>
+        <v>97</v>
+      </c>
+      <c r="N76" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="O76" s="15" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="77" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I77" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J77" s="14" t="s">
-        <v>99</v>
+        <v>72</v>
+      </c>
+      <c r="N77" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="O77" s="15" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="78" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I78" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J78" s="14" t="s">
-        <v>100</v>
+        <v>52</v>
+      </c>
+      <c r="N78" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="O78" s="15" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="79" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I79" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J79" s="14" t="s">
-        <v>30</v>
+        <v>43</v>
+      </c>
+      <c r="N79" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="O79" s="15" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="80" spans="9:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I80" s="8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="J80" s="14" t="s">
-        <v>101</v>
+        <v>30</v>
+      </c>
+      <c r="N80" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="O80" s="15" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="81" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I81" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J81" s="14" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="82" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I82" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J82" s="14" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="83" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I83" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="J83" s="14" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="84" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I84" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="J84" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="85" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I85" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="J83" s="14" t="s">
+      <c r="J85" s="14" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="86" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I86" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J86" s="14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="87" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I87" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J87" s="14" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="88" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I88" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J88" s="14" t="s">
         <v>30</v>
-      </c>
-    </row>
-    <row r="84" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I84" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="J84" s="13" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="85" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I85" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="J85" s="13" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="86" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I86" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="J86" s="13" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="87" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I87" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="J87" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="88" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I88" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="J88" s="13" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="89" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I89" s="12" t="s">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="J89" s="13" t="s">
-        <v>122</v>
+        <v>90</v>
       </c>
     </row>
     <row r="90" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I90" s="12" t="s">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="J90" s="13" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="91" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I91" s="12" t="s">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="J91" s="13" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="92" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I92" s="12" t="s">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="J92" s="13" t="s">
         <v>30</v>
@@ -7990,209 +8118,249 @@
     </row>
     <row r="93" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I93" s="12" t="s">
-        <v>44</v>
+        <v>120</v>
       </c>
       <c r="J93" s="13" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="94" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I94" s="12" t="s">
-        <v>44</v>
+        <v>120</v>
       </c>
       <c r="J94" s="13" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="95" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I95" s="12" t="s">
-        <v>44</v>
+        <v>120</v>
       </c>
       <c r="J95" s="13" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="96" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I96" s="12" t="s">
-        <v>44</v>
+        <v>120</v>
       </c>
       <c r="J96" s="13" t="s">
-        <v>30</v>
+        <v>124</v>
       </c>
     </row>
     <row r="97" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I97" s="12" t="s">
-        <v>45</v>
+        <v>120</v>
       </c>
       <c r="J97" s="13" t="s">
-        <v>128</v>
+        <v>30</v>
       </c>
     </row>
     <row r="98" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I98" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J98" s="13" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="99" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I99" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J99" s="13" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="100" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I100" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="J100" s="13" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="101" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I101" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="J101" s="13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="102" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I102" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="J100" s="13" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="101" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I101" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="J101" s="15" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="102" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I102" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="J102" s="15" t="s">
-        <v>108</v>
+      <c r="J102" s="13" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="103" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I103" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="J103" s="15" t="s">
-        <v>109</v>
+      <c r="I103" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="J103" s="13" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="104" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I104" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="J104" s="15" t="s">
-        <v>110</v>
+      <c r="I104" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="J104" s="13" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="105" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="I105" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="J105" s="15" t="s">
+      <c r="I105" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="J105" s="13" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="106" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I106" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J106" s="15" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="107" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I107" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J107" s="15" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="108" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I108" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J108" s="15" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="109" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I109" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J109" s="15" t="s">
-        <v>30</v>
+        <v>110</v>
       </c>
     </row>
     <row r="110" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I110" s="15" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="J110" s="15" t="s">
-        <v>114</v>
+        <v>30</v>
       </c>
     </row>
     <row r="111" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I111" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J111" s="15" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="112" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I112" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J112" s="15" t="s">
-        <v>30</v>
+        <v>112</v>
       </c>
     </row>
     <row r="113" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I113" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J113" s="15" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="114" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I114" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="J114" s="15" t="s">
-        <v>117</v>
+        <v>30</v>
       </c>
     </row>
     <row r="115" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I115" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J115" s="15" t="s">
-        <v>30</v>
+        <v>114</v>
       </c>
     </row>
     <row r="116" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I116" s="15" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="J116" s="15" t="s">
-        <v>141</v>
+        <v>115</v>
       </c>
     </row>
     <row r="117" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I117" s="15" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="J117" s="15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="118" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I118" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="J118" s="15" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="119" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I119" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="J119" s="15" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="120" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I120" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="J120" s="15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="121" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I121" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="J118" s="15" t="s">
+      <c r="J121" s="15" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="122" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I122" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="J122" s="15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="123" spans="9:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="I123" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="J123" s="15" t="s">
         <v>30</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: ajustes minha conta, suporte, modelos cartao de creditoe conta corrente
</commit_message>
<xml_diff>
--- a/public/modelo_importacao_cartao-credito.xlsx
+++ b/public/modelo_importacao_cartao-credito.xlsx
@@ -585,10 +585,10 @@
     <t>Itaú</t>
   </si>
   <si>
-    <t>Prestação Apartamento</t>
-  </si>
-  <si>
     <t>Maio/2026</t>
+  </si>
+  <si>
+    <t>Reforma Apartamento</t>
   </si>
 </sst>
 </file>
@@ -1308,7 +1308,7 @@
         <v>46113</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G5" s="21" t="s">
         <v>168</v>
@@ -1355,7 +1355,7 @@
         <v>167</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H6" s="19" t="s">
         <v>169</v>

</xml_diff>